<commit_message>
RC duplicates xlsx: keep the hand-made ArmSoft goods, delete our imported ones (user)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/final/royal-canin-armsoft-duplicates.xlsx
+++ b/final/royal-canin-armsoft-duplicates.xlsx
@@ -452,22 +452,22 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Duplicate code (hand-made)</t>
+          <t>KEEP code (hand-made, has the invoices)</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Duplicate name in ArmSoft</t>
+          <t>KEEP: name in ArmSoft</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Keep code</t>
+          <t>DELETE code (our import)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Keep: name in ArmSoft</t>
+          <t>DELETE: name in ArmSoft</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -477,7 +477,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Keep: barcode / PLU</t>
+          <t>Barcode / PLU to move onto the KEEP code</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -549,7 +549,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Move any stock from the duplicate to the keep code, then retire the duplicate</t>
+          <t>Delete the DELETE code; then put its barcode/PLU on the KEEP code (a barcode can only be on one good)</t>
         </is>
       </c>
     </row>
@@ -601,7 +601,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Move any stock from the duplicate to the keep code, then retire the duplicate</t>
+          <t>Delete the DELETE code; then put its barcode/PLU on the KEEP code (a barcode can only be on one good)</t>
         </is>
       </c>
     </row>
@@ -653,7 +653,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Move any stock from the duplicate to the keep code, then retire the duplicate</t>
+          <t>Delete the DELETE code; then put its barcode/PLU on the KEEP code (a barcode can only be on one good)</t>
         </is>
       </c>
     </row>
@@ -705,7 +705,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Move any stock from the duplicate to the keep code, then retire the duplicate</t>
+          <t>Delete the DELETE code; then put its barcode/PLU on the KEEP code (a barcode can only be on one good)</t>
         </is>
       </c>
     </row>
@@ -757,7 +757,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Move any stock from the duplicate to the keep code, then retire the duplicate</t>
+          <t>Delete the DELETE code; then put its barcode/PLU on the KEEP code (a barcode can only be on one good)</t>
         </is>
       </c>
     </row>
@@ -809,7 +809,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Move any stock from the duplicate to the keep code, then retire the duplicate</t>
+          <t>Delete the DELETE code; then put its barcode/PLU on the KEEP code (a barcode can only be on one good)</t>
         </is>
       </c>
     </row>
@@ -861,7 +861,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Move any stock from the duplicate to the keep code, then retire the duplicate</t>
+          <t>Delete the DELETE code; then put its barcode/PLU on the KEEP code (a barcode can only be on one good)</t>
         </is>
       </c>
     </row>
@@ -913,7 +913,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Move any stock from the duplicate to the keep code, then retire the duplicate</t>
+          <t>Delete the DELETE code; then put its barcode/PLU on the KEEP code (a barcode can only be on one good)</t>
         </is>
       </c>
     </row>
@@ -965,7 +965,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Move any stock from the duplicate to the keep code, then retire the duplicate</t>
+          <t>Delete the DELETE code; then put its barcode/PLU on the KEEP code (a barcode can only be on one good)</t>
         </is>
       </c>
     </row>
@@ -1017,7 +1017,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Move any stock from the duplicate to the keep code, then retire the duplicate</t>
+          <t>Delete the DELETE code; then put its barcode/PLU on the KEEP code (a barcode can only be on one good)</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1069,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Move any stock from the duplicate to the keep code, then retire the duplicate</t>
+          <t>Delete the DELETE code; then put its barcode/PLU on the KEEP code (a barcode can only be on one good)</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1121,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Move any stock from the duplicate to the keep code, then retire the duplicate</t>
+          <t>Delete the DELETE code; then put its barcode/PLU on the KEEP code (a barcode can only be on one good)</t>
         </is>
       </c>
     </row>
@@ -1173,7 +1173,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Move any stock from the duplicate to the keep code, then retire the duplicate</t>
+          <t>Delete the DELETE code; then put its barcode/PLU on the KEEP code (a barcode can only be on one good)</t>
         </is>
       </c>
     </row>
@@ -1225,7 +1225,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Move any stock from the duplicate to the keep code, then retire the duplicate</t>
+          <t>Delete the DELETE code; then put its barcode/PLU on the KEEP code (a barcode can only be on one good)</t>
         </is>
       </c>
     </row>
@@ -1277,7 +1277,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Move any stock from the duplicate to the keep code, then retire the duplicate</t>
+          <t>Delete the DELETE code; then put its barcode/PLU on the KEEP code (a barcode can only be on one good)</t>
         </is>
       </c>
     </row>
@@ -1329,7 +1329,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Move any stock from the duplicate to the keep code, then retire the duplicate</t>
+          <t>Delete the DELETE code; then put its barcode/PLU on the KEEP code (a barcode can only be on one good)</t>
         </is>
       </c>
     </row>
@@ -1381,7 +1381,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Move any stock from the duplicate to the keep code, then retire the duplicate</t>
+          <t>Delete the DELETE code; then put its barcode/PLU on the KEEP code (a barcode can only be on one good)</t>
         </is>
       </c>
     </row>
@@ -1433,7 +1433,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Move any stock from the duplicate to the keep code, then retire the duplicate</t>
+          <t>Delete the DELETE code; then put its barcode/PLU on the KEEP code (a barcode can only be on one good)</t>
         </is>
       </c>
     </row>
@@ -1485,7 +1485,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Move any stock from the duplicate to the keep code, then retire the duplicate</t>
+          <t>Delete the DELETE code; then put its barcode/PLU on the KEEP code (a barcode can only be on one good)</t>
         </is>
       </c>
     </row>
@@ -1537,7 +1537,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Move any stock from the duplicate to the keep code, then retire the duplicate</t>
+          <t>Delete the DELETE code; then put its barcode/PLU on the KEEP code (a barcode can only be on one good)</t>
         </is>
       </c>
     </row>
@@ -1589,7 +1589,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Move any stock from the duplicate to the keep code, then retire the duplicate</t>
+          <t>Delete the DELETE code; then put its barcode/PLU on the KEEP code (a barcode can only be on one good)</t>
         </is>
       </c>
     </row>
@@ -1641,7 +1641,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Move any stock from the duplicate to the keep code, then retire the duplicate</t>
+          <t>Delete the DELETE code; then put its barcode/PLU on the KEEP code (a barcode can only be on one good)</t>
         </is>
       </c>
     </row>
@@ -1693,7 +1693,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Move any stock from the duplicate to the keep code, then retire the duplicate</t>
+          <t>Delete the DELETE code; then put its barcode/PLU on the KEEP code (a barcode can only be on one good)</t>
         </is>
       </c>
     </row>
@@ -1738,10 +1738,9 @@
           <t>sure</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Move any stock from the duplicate to the keep code, then retire the duplicate</t>
+          <t>Delete the DELETE code; then put its barcode/PLU on the KEEP code (a barcode can only be on one good)</t>
         </is>
       </c>
     </row>
@@ -1793,7 +1792,7 @@
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>Move any stock from the duplicate to the keep code, then retire the duplicate</t>
+          <t>Delete the DELETE code; then put its barcode/PLU on the KEEP code (a barcode can only be on one good)</t>
         </is>
       </c>
     </row>
@@ -1838,10 +1837,9 @@
           <t>sure</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Move any stock from the duplicate to the keep code, then retire the duplicate</t>
+          <t>Delete the DELETE code; then put its barcode/PLU on the KEEP code (a barcode can only be on one good)</t>
         </is>
       </c>
     </row>
@@ -1893,7 +1891,7 @@
       </c>
       <c r="J28" s="4" t="inlineStr">
         <is>
-          <t>Move any stock from the duplicate to the keep code, then retire the duplicate</t>
+          <t>Delete the DELETE code; then put its barcode/PLU on the KEEP code (a barcode can only be on one good)</t>
         </is>
       </c>
     </row>
@@ -1938,10 +1936,9 @@
           <t>sure</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Move any stock from the duplicate to the keep code, then retire the duplicate</t>
+          <t>Delete the DELETE code; then put its barcode/PLU on the KEEP code (a barcode can only be on one good)</t>
         </is>
       </c>
     </row>
@@ -1993,7 +1990,7 @@
       </c>
       <c r="J30" s="4" t="inlineStr">
         <is>
-          <t>Move any stock from the duplicate to the keep code, then retire the duplicate</t>
+          <t>Delete the DELETE code; then put its barcode/PLU on the KEEP code (a barcode can only be on one good)</t>
         </is>
       </c>
     </row>
@@ -2038,10 +2035,9 @@
           <t>sure</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Move any stock from the duplicate to the keep code, then retire the duplicate</t>
+          <t>Delete the DELETE code; then put its barcode/PLU on the KEEP code (a barcode can only be on one good)</t>
         </is>
       </c>
     </row>

</xml_diff>